<commit_message>
Templates: strip data-validation dropdowns from header row 2 (all BU)
Factory/CLAIM/etc list validations bled into header cells (S2/N2/O2/B2/C2/H2/W2/AA2),
so headers like %CLAIM showed a stray G1..G4 dropdown. Bump every row-2 range to row 3
and drop stray single header cells; remove a validation that became empty (EA).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/air-request-template_EA.xlsx
+++ b/public/air-request-template_EA.xlsx
@@ -10927,23 +10927,20 @@
     <mergeCell ref="O1:Q1"/>
     <mergeCell ref="R1:AC1"/>
   </mergeCells>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2 N2" xr:uid="{00000000-0002-0000-0000-000008000000}">
-      <formula1>INDIRECT("MASTER_FACT[G]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2 N3:N1048576" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1048576" xr:uid="{00000000-0002-0000-0000-00000B000000}">
       <formula1>INDIRECT("MASTER_COUNTRY[SHIPTO_COUNTRY]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W282 Z3:Z1048576 V3:V282 R3:R1048576 AA2:AA1048576 V283:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W3:W282 Z3:Z1048576 V3:V282 R3:R1048576 AA3:AA1048576 V283:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT("MASTER_CLAIM[CLAIM]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>INDIRECT("MASTER_BRAND[BRAND_NAME]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:C1048576" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>INDIRECT("MASTER_BU[BU]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H1048576" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>INDIRECT("MASTER_GARMENT_TYPE[DESCRIPTION]")</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>